<commit_message>
signal-book WIP: KYN-KJT/KYN-KSRA data updates, plan + successor notes
Working data spreadsheets for KYN-KJT and KYN-KSRA sections, master-plan
and unresolved-successor notes, and a render cleanup (drop dead CSS rule).
Recovered from the mixed WIP that was auto-stashed on 2026-07-02; the
loco-link roster and signal-sighting parts of that stash live on their
own feature branches now.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/KYN_KJT/dnse_signals.xlsx
+++ b/data/KYN_KJT/dnse_signals.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y61"/>
+  <dimension ref="A1:Y62"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -502,7 +502,7 @@
         <v>53.262</v>
       </c>
       <c r="I2" t="str">
-        <v>Manual</v>
+        <v>Semi-Automatic</v>
       </c>
       <c r="J2" t="str">
         <v>Right</v>
@@ -546,10 +546,16 @@
       <c r="W2">
         <v>1</v>
       </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>KYN S-82</v>
+        <v>KYN S-58</v>
       </c>
       <c r="B3" t="str">
         <v>KYN</v>
@@ -567,13 +573,13 @@
         <v>DN</v>
       </c>
       <c r="G3" t="str">
-        <v>54/26</v>
-      </c>
-      <c r="H3">
-        <v>54.451</v>
+        <v>PF-5 STR</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
       </c>
       <c r="I3" t="str">
-        <v>Manual</v>
+        <v>Semi-Automatic</v>
       </c>
       <c r="J3" t="str">
         <v>Left</v>
@@ -603,24 +609,36 @@
         <v>0</v>
       </c>
       <c r="S3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T3">
         <v>0</v>
       </c>
+      <c r="U3" t="str">
+        <v>RI:L1=S-72</v>
+      </c>
+      <c r="V3" t="str">
+        <v>Book shows one left arm on top of vertical stem</v>
+      </c>
       <c r="W3">
         <v>1</v>
       </c>
       <c r="X3" t="str">
-        <v>54/26</v>
-      </c>
-      <c r="Y3">
-        <v>350</v>
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>SE-5511</v>
+        <v>KYN S-82</v>
+      </c>
+      <c r="B4" t="str">
+        <v>KYN</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Kalyan</v>
       </c>
       <c r="D4" t="str">
         <v>KYN-KJT</v>
@@ -632,13 +650,13 @@
         <v>DN</v>
       </c>
       <c r="G4" t="str">
-        <v>55/28</v>
+        <v>54/26</v>
       </c>
       <c r="H4">
-        <v>55.412</v>
+        <v>54.451</v>
       </c>
       <c r="I4" t="str">
-        <v>Automatic</v>
+        <v>Semi-Automatic</v>
       </c>
       <c r="J4" t="str">
         <v>Left</v>
@@ -673,19 +691,31 @@
       <c r="T4">
         <v>0</v>
       </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
       <c r="W4">
         <v>1</v>
       </c>
       <c r="X4" t="str">
-        <v>55/28</v>
+        <v>54/26</v>
       </c>
       <c r="Y4">
-        <v>400</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>SE-5609</v>
+        <v>SE-5511</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
       </c>
       <c r="D5" t="str">
         <v>KYN-KJT</v>
@@ -697,10 +727,10 @@
         <v>DN</v>
       </c>
       <c r="G5" t="str">
-        <v>56/28</v>
+        <v>55/28</v>
       </c>
       <c r="H5">
-        <v>56.568</v>
+        <v>55.412</v>
       </c>
       <c r="I5" t="str">
         <v>Automatic</v>
@@ -738,19 +768,31 @@
       <c r="T5">
         <v>0</v>
       </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
       <c r="W5">
         <v>1</v>
       </c>
       <c r="X5" t="str">
-        <v>56/28</v>
+        <v>55/28</v>
       </c>
       <c r="Y5">
-        <v>350</v>
+        <v>400</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SE-5707</v>
+        <v>SE-5609</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
       </c>
       <c r="D6" t="str">
         <v>KYN-KJT</v>
@@ -762,10 +804,10 @@
         <v>DN</v>
       </c>
       <c r="G6" t="str">
-        <v>57/24</v>
+        <v>56/28</v>
       </c>
       <c r="H6">
-        <v>57.326</v>
+        <v>56.568</v>
       </c>
       <c r="I6" t="str">
         <v>Automatic</v>
@@ -774,7 +816,7 @@
         <v>Left</v>
       </c>
       <c r="K6" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="L6">
         <v>0</v>
@@ -803,19 +845,31 @@
       <c r="T6">
         <v>0</v>
       </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
       <c r="W6">
         <v>1</v>
       </c>
       <c r="X6" t="str">
-        <v>57/24</v>
+        <v>56/28</v>
       </c>
       <c r="Y6">
-        <v>250</v>
+        <v>350</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Gate-4</v>
+        <v>SE-5707</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
       </c>
       <c r="D7" t="str">
         <v>KYN-KJT</v>
@@ -827,19 +881,19 @@
         <v>DN</v>
       </c>
       <c r="G7" t="str">
-        <v>58/26</v>
+        <v>57/24</v>
       </c>
       <c r="H7">
-        <v>58.471000000000004</v>
+        <v>57.326</v>
       </c>
       <c r="I7" t="str">
-        <v>Gate</v>
+        <v>Automatic</v>
       </c>
       <c r="J7" t="str">
         <v>Left</v>
       </c>
       <c r="K7" t="str">
-        <v>Unknown</v>
+        <v>Right</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -868,25 +922,31 @@
       <c r="T7">
         <v>0</v>
       </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
       <c r="W7">
         <v>1</v>
       </c>
       <c r="X7" t="str">
-        <v>58/26</v>
+        <v>57/24</v>
       </c>
       <c r="Y7">
-        <v>350</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ABH S-2</v>
+        <v>Gate-4</v>
       </c>
       <c r="B8" t="str">
-        <v>ABH</v>
+        <v/>
       </c>
       <c r="C8" t="str">
-        <v>Ambernath</v>
+        <v/>
       </c>
       <c r="D8" t="str">
         <v>KYN-KJT</v>
@@ -898,19 +958,19 @@
         <v>DN</v>
       </c>
       <c r="G8" t="str">
-        <v>59/4</v>
+        <v>58/26</v>
       </c>
       <c r="H8">
-        <v>59.015</v>
+        <v>58.471000000000004</v>
       </c>
       <c r="I8" t="str">
-        <v>Manual</v>
+        <v>Gate</v>
       </c>
       <c r="J8" t="str">
         <v>Left</v>
       </c>
       <c r="K8" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="L8">
         <v>0</v>
@@ -928,7 +988,7 @@
         <v>0</v>
       </c>
       <c r="Q8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R8">
         <v>0</v>
@@ -937,27 +997,27 @@
         <v>0</v>
       </c>
       <c r="T8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U8" t="str">
-        <v>RI: R1=PF-2; R2=PF-3</v>
+        <v/>
       </c>
       <c r="V8" t="str">
-        <v>Book shows two right arms on top of vertical stem</v>
+        <v/>
       </c>
       <c r="W8">
         <v>1</v>
       </c>
       <c r="X8" t="str">
-        <v>59/4</v>
+        <v>58/26</v>
       </c>
       <c r="Y8">
-        <v>300</v>
+        <v>350</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ABH S-6</v>
+        <v>ABH S-2</v>
       </c>
       <c r="B9" t="str">
         <v>ABH</v>
@@ -975,10 +1035,10 @@
         <v>DN</v>
       </c>
       <c r="G9" t="str">
-        <v>PF-1 STR</v>
+        <v>59/4</v>
       </c>
       <c r="H9">
-        <v>59.795</v>
+        <v>59.015</v>
       </c>
       <c r="I9" t="str">
         <v>Manual</v>
@@ -987,7 +1047,7 @@
         <v>Left</v>
       </c>
       <c r="K9" t="str">
-        <v>Unknown</v>
+        <v>Right</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -1008,30 +1068,33 @@
         <v>1</v>
       </c>
       <c r="R9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U9" t="str">
-        <v>RI: L1=DN LL</v>
+        <v>RI: R1=PF-2; R2=PF-3</v>
       </c>
       <c r="V9" t="str">
-        <v>Book shows one left arm on top of vertical stem</v>
+        <v>Book shows two right arms on top of vertical stem</v>
       </c>
       <c r="W9">
         <v>1</v>
       </c>
+      <c r="X9" t="str">
+        <v>59/4</v>
+      </c>
       <c r="Y9">
-        <v>400</v>
+        <v>300</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ABH S-15</v>
+        <v>ABH S-6</v>
       </c>
       <c r="B10" t="str">
         <v>ABH</v>
@@ -1049,13 +1112,13 @@
         <v>DN</v>
       </c>
       <c r="G10" t="str">
-        <v>60/32</v>
+        <v>PF-1 STR</v>
       </c>
       <c r="H10">
-        <v>60.702</v>
+        <v>59.795</v>
       </c>
       <c r="I10" t="str">
-        <v>Semi-Automatic</v>
+        <v>Manual</v>
       </c>
       <c r="J10" t="str">
         <v>Left</v>
@@ -1079,30 +1142,36 @@
         <v>0</v>
       </c>
       <c r="Q10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T10">
         <v>0</v>
       </c>
+      <c r="U10" t="str">
+        <v>RI: L1=DN LL</v>
+      </c>
+      <c r="V10" t="str">
+        <v>Book shows one left arm on top of vertical stem</v>
+      </c>
       <c r="W10">
         <v>1</v>
       </c>
       <c r="X10" t="str">
-        <v>60/32</v>
+        <v/>
       </c>
       <c r="Y10">
-        <v>800</v>
+        <v>400</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ABH S-18</v>
+        <v>ABH S-15</v>
       </c>
       <c r="B11" t="str">
         <v>ABH</v>
@@ -1120,10 +1189,10 @@
         <v>DN</v>
       </c>
       <c r="G11" t="str">
-        <v>61/20</v>
+        <v>60/32</v>
       </c>
       <c r="H11">
-        <v>61.442</v>
+        <v>60.702</v>
       </c>
       <c r="I11" t="str">
         <v>Semi-Automatic</v>
@@ -1132,7 +1201,7 @@
         <v>Left</v>
       </c>
       <c r="K11" t="str">
-        <v>Left</v>
+        <v>Unknown</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -1161,19 +1230,31 @@
       <c r="T11">
         <v>0</v>
       </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v/>
+      </c>
       <c r="W11">
         <v>1</v>
       </c>
       <c r="X11" t="str">
-        <v>61/20</v>
+        <v>60/32</v>
       </c>
       <c r="Y11">
-        <v>350</v>
+        <v>800</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>SE-6205</v>
+        <v>ABH S-18</v>
+      </c>
+      <c r="B12" t="str">
+        <v>ABH</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Ambernath</v>
       </c>
       <c r="D12" t="str">
         <v>KYN-KJT</v>
@@ -1185,19 +1266,19 @@
         <v>DN</v>
       </c>
       <c r="G12" t="str">
-        <v>62/10</v>
+        <v>61/20</v>
       </c>
       <c r="H12">
-        <v>62.168</v>
+        <v>61.442</v>
       </c>
       <c r="I12" t="str">
-        <v>Automatic</v>
+        <v>Semi-Automatic</v>
       </c>
       <c r="J12" t="str">
         <v>Left</v>
       </c>
       <c r="K12" t="str">
-        <v>Unknown</v>
+        <v>Left</v>
       </c>
       <c r="L12">
         <v>0</v>
@@ -1226,19 +1307,31 @@
       <c r="T12">
         <v>0</v>
       </c>
+      <c r="U12" t="str">
+        <v/>
+      </c>
+      <c r="V12" t="str">
+        <v/>
+      </c>
       <c r="W12">
         <v>1</v>
       </c>
       <c r="X12" t="str">
-        <v>62/10</v>
+        <v>61/20</v>
       </c>
       <c r="Y12">
-        <v>550</v>
+        <v>350</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Gate-7</v>
+        <v>SE-6205</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v/>
       </c>
       <c r="D13" t="str">
         <v>KYN-KJT</v>
@@ -1250,19 +1343,19 @@
         <v>DN</v>
       </c>
       <c r="G13" t="str">
-        <v>63/18</v>
+        <v>62/10</v>
       </c>
       <c r="H13">
-        <v>63.146</v>
+        <v>62.168</v>
       </c>
       <c r="I13" t="str">
-        <v>Gate</v>
+        <v>Automatic</v>
       </c>
       <c r="J13" t="str">
         <v>Left</v>
       </c>
       <c r="K13" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="L13">
         <v>0</v>
@@ -1291,19 +1384,31 @@
       <c r="T13">
         <v>0</v>
       </c>
+      <c r="U13" t="str">
+        <v/>
+      </c>
+      <c r="V13" t="str">
+        <v/>
+      </c>
       <c r="W13">
         <v>1</v>
       </c>
       <c r="X13" t="str">
-        <v>63/18</v>
+        <v>62/10</v>
       </c>
       <c r="Y13">
-        <v>300</v>
+        <v>550</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SE-6315</v>
+        <v>Gate-7</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v/>
       </c>
       <c r="D14" t="str">
         <v>KYN-KJT</v>
@@ -1315,19 +1420,19 @@
         <v>DN</v>
       </c>
       <c r="G14" t="str">
-        <v>63/44</v>
+        <v>63/18</v>
       </c>
       <c r="H14">
-        <v>63.836</v>
+        <v>63.146</v>
       </c>
       <c r="I14" t="str">
-        <v>Automatic</v>
+        <v>Gate</v>
       </c>
       <c r="J14" t="str">
         <v>Left</v>
       </c>
       <c r="K14" t="str">
-        <v>Left</v>
+        <v>Right</v>
       </c>
       <c r="L14">
         <v>0</v>
@@ -1356,19 +1461,31 @@
       <c r="T14">
         <v>0</v>
       </c>
+      <c r="U14" t="str">
+        <v/>
+      </c>
+      <c r="V14" t="str">
+        <v/>
+      </c>
       <c r="W14">
         <v>1</v>
       </c>
       <c r="X14" t="str">
-        <v>63/44</v>
+        <v>63/18</v>
       </c>
       <c r="Y14">
-        <v>400</v>
+        <v>300</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SE-6411</v>
+        <v>SE-6315</v>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v/>
       </c>
       <c r="D15" t="str">
         <v>KYN-KJT</v>
@@ -1380,10 +1497,10 @@
         <v>DN</v>
       </c>
       <c r="G15" t="str">
-        <v>64/24</v>
+        <v>63/44</v>
       </c>
       <c r="H15">
-        <v>64.536</v>
+        <v>63.836</v>
       </c>
       <c r="I15" t="str">
         <v>Automatic</v>
@@ -1392,7 +1509,7 @@
         <v>Left</v>
       </c>
       <c r="K15" t="str">
-        <v>Right</v>
+        <v>Left</v>
       </c>
       <c r="L15">
         <v>0</v>
@@ -1421,19 +1538,31 @@
       <c r="T15">
         <v>0</v>
       </c>
+      <c r="U15" t="str">
+        <v/>
+      </c>
+      <c r="V15" t="str">
+        <v/>
+      </c>
       <c r="W15">
         <v>1</v>
       </c>
       <c r="X15" t="str">
-        <v>64/24</v>
+        <v>63/44</v>
       </c>
       <c r="Y15">
-        <v>500</v>
+        <v>400</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SE-6513</v>
+        <v>SE-6411</v>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
       </c>
       <c r="D16" t="str">
         <v>KYN-KJT</v>
@@ -1445,10 +1574,10 @@
         <v>DN</v>
       </c>
       <c r="G16" t="str">
-        <v>65/14</v>
+        <v>64/24</v>
       </c>
       <c r="H16">
-        <v>65.211</v>
+        <v>64.536</v>
       </c>
       <c r="I16" t="str">
         <v>Automatic</v>
@@ -1457,7 +1586,7 @@
         <v>Left</v>
       </c>
       <c r="K16" t="str">
-        <v>Left</v>
+        <v>Right</v>
       </c>
       <c r="L16">
         <v>0</v>
@@ -1486,19 +1615,31 @@
       <c r="T16">
         <v>0</v>
       </c>
+      <c r="U16" t="str">
+        <v/>
+      </c>
+      <c r="V16" t="str">
+        <v/>
+      </c>
       <c r="W16">
         <v>1</v>
       </c>
       <c r="X16" t="str">
-        <v>65/14</v>
+        <v>64/24</v>
       </c>
       <c r="Y16">
-        <v>450</v>
+        <v>500</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SE-6515</v>
+        <v>SE-6513</v>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v/>
       </c>
       <c r="D17" t="str">
         <v>KYN-KJT</v>
@@ -1510,10 +1651,10 @@
         <v>DN</v>
       </c>
       <c r="G17" t="str">
-        <v>65/40</v>
+        <v>65/14</v>
       </c>
       <c r="H17">
-        <v>65.837</v>
+        <v>65.211</v>
       </c>
       <c r="I17" t="str">
         <v>Automatic</v>
@@ -1522,7 +1663,7 @@
         <v>Left</v>
       </c>
       <c r="K17" t="str">
-        <v>Right</v>
+        <v>Left</v>
       </c>
       <c r="L17">
         <v>0</v>
@@ -1551,25 +1692,31 @@
       <c r="T17">
         <v>0</v>
       </c>
+      <c r="U17" t="str">
+        <v/>
+      </c>
+      <c r="V17" t="str">
+        <v/>
+      </c>
       <c r="W17">
         <v>1</v>
       </c>
       <c r="X17" t="str">
-        <v>65/40</v>
+        <v>65/14</v>
       </c>
       <c r="Y17">
-        <v>500</v>
+        <v>450</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>BUD S-2</v>
+        <v>SE-6515</v>
       </c>
       <c r="B18" t="str">
-        <v>BUD</v>
+        <v/>
       </c>
       <c r="C18" t="str">
-        <v>Badlapur</v>
+        <v/>
       </c>
       <c r="D18" t="str">
         <v>KYN-KJT</v>
@@ -1581,19 +1728,19 @@
         <v>DN</v>
       </c>
       <c r="G18" t="str">
-        <v>66/22</v>
+        <v>65/40</v>
       </c>
       <c r="H18">
-        <v>66.417</v>
+        <v>65.837</v>
       </c>
       <c r="I18" t="str">
-        <v>Manual</v>
+        <v>Automatic</v>
       </c>
       <c r="J18" t="str">
         <v>Left</v>
       </c>
       <c r="K18" t="str">
-        <v>Left</v>
+        <v>Right</v>
       </c>
       <c r="L18">
         <v>0</v>
@@ -1611,28 +1758,28 @@
         <v>0</v>
       </c>
       <c r="Q18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R18">
         <v>0</v>
       </c>
       <c r="S18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T18">
         <v>0</v>
       </c>
       <c r="U18" t="str">
-        <v>RI: L1=PF-1</v>
+        <v/>
       </c>
       <c r="V18" t="str">
-        <v>Book shows one left arm on top of vertical stem</v>
+        <v/>
       </c>
       <c r="W18">
         <v>1</v>
       </c>
       <c r="X18" t="str">
-        <v>66/22</v>
+        <v>65/40</v>
       </c>
       <c r="Y18">
         <v>500</v>
@@ -1640,7 +1787,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>BUD S-9</v>
+        <v>BUD S-2</v>
       </c>
       <c r="B19" t="str">
         <v>BUD</v>
@@ -1658,10 +1805,10 @@
         <v>DN</v>
       </c>
       <c r="G19" t="str">
-        <v>PF-2 STR</v>
+        <v>66/22</v>
       </c>
       <c r="H19">
-        <v>67.382</v>
+        <v>66.417</v>
       </c>
       <c r="I19" t="str">
         <v>Manual</v>
@@ -1670,7 +1817,7 @@
         <v>Left</v>
       </c>
       <c r="K19" t="str">
-        <v>Unknown</v>
+        <v>Left</v>
       </c>
       <c r="L19">
         <v>0</v>
@@ -1691,7 +1838,7 @@
         <v>1</v>
       </c>
       <c r="R19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S19">
         <v>1</v>
@@ -1700,7 +1847,7 @@
         <v>0</v>
       </c>
       <c r="U19" t="str">
-        <v>RI: L1=DN LL</v>
+        <v>RI: L1=PF-1</v>
       </c>
       <c r="V19" t="str">
         <v>Book shows one left arm on top of vertical stem</v>
@@ -1708,13 +1855,16 @@
       <c r="W19">
         <v>1</v>
       </c>
+      <c r="X19" t="str">
+        <v>66/22</v>
+      </c>
       <c r="Y19">
-        <v>400</v>
+        <v>500</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>BUD S-12</v>
+        <v>BUD S-9</v>
       </c>
       <c r="B20" t="str">
         <v>BUD</v>
@@ -1732,10 +1882,10 @@
         <v>DN</v>
       </c>
       <c r="G20" t="str">
-        <v>68/32</v>
+        <v>PF-2 STR</v>
       </c>
       <c r="H20">
-        <v>68.531</v>
+        <v>67.382</v>
       </c>
       <c r="I20" t="str">
         <v>Manual</v>
@@ -1744,7 +1894,7 @@
         <v>Left</v>
       </c>
       <c r="K20" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="L20">
         <v>0</v>
@@ -1762,30 +1912,36 @@
         <v>0</v>
       </c>
       <c r="Q20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T20">
         <v>0</v>
       </c>
+      <c r="U20" t="str">
+        <v>RI: L1=DN LL</v>
+      </c>
+      <c r="V20" t="str">
+        <v>Book shows one left arm on top of vertical stem</v>
+      </c>
       <c r="W20">
         <v>1</v>
       </c>
       <c r="X20" t="str">
-        <v>68/32</v>
+        <v/>
       </c>
       <c r="Y20">
-        <v>550</v>
+        <v>400</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>BUD S-14</v>
+        <v>BUD S-12</v>
       </c>
       <c r="B21" t="str">
         <v>BUD</v>
@@ -1803,19 +1959,19 @@
         <v>DN</v>
       </c>
       <c r="G21" t="str">
-        <v>68/50</v>
+        <v>68/32</v>
       </c>
       <c r="H21">
-        <v>68.889</v>
+        <v>68.531</v>
       </c>
       <c r="I21" t="str">
-        <v>Semi-Automatic</v>
+        <v>Manual</v>
       </c>
       <c r="J21" t="str">
         <v>Left</v>
       </c>
       <c r="K21" t="str">
-        <v>Unknown</v>
+        <v>Right</v>
       </c>
       <c r="L21">
         <v>0</v>
@@ -1844,19 +2000,31 @@
       <c r="T21">
         <v>0</v>
       </c>
+      <c r="U21" t="str">
+        <v/>
+      </c>
+      <c r="V21" t="str">
+        <v/>
+      </c>
       <c r="W21">
         <v>1</v>
       </c>
       <c r="X21" t="str">
-        <v>68/50</v>
+        <v>68/32</v>
       </c>
       <c r="Y21">
-        <v>400</v>
+        <v>550</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SE-6913</v>
+        <v>BUD S-14</v>
+      </c>
+      <c r="B22" t="str">
+        <v>BUD</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Badlapur</v>
       </c>
       <c r="D22" t="str">
         <v>KYN-KJT</v>
@@ -1868,19 +2036,19 @@
         <v>DN</v>
       </c>
       <c r="G22" t="str">
-        <v>69/36</v>
+        <v>68/50</v>
       </c>
       <c r="H22">
-        <v>69.769</v>
+        <v>68.889</v>
       </c>
       <c r="I22" t="str">
-        <v>Automatic</v>
+        <v>Semi-Automatic</v>
       </c>
       <c r="J22" t="str">
         <v>Left</v>
       </c>
       <c r="K22" t="str">
-        <v>Left</v>
+        <v>Unknown</v>
       </c>
       <c r="L22">
         <v>0</v>
@@ -1909,19 +2077,31 @@
       <c r="T22">
         <v>0</v>
       </c>
+      <c r="U22" t="str">
+        <v/>
+      </c>
+      <c r="V22" t="str">
+        <v/>
+      </c>
       <c r="W22">
         <v>1</v>
       </c>
       <c r="X22" t="str">
-        <v>69/36</v>
+        <v>68/50</v>
       </c>
       <c r="Y22">
-        <v>300</v>
+        <v>400</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SE-7013</v>
+        <v>SE-6913</v>
+      </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
+        <v/>
       </c>
       <c r="D23" t="str">
         <v>KYN-KJT</v>
@@ -1933,10 +2113,10 @@
         <v>DN</v>
       </c>
       <c r="G23" t="str">
-        <v>70/34</v>
+        <v>69/36</v>
       </c>
       <c r="H23">
-        <v>70.719</v>
+        <v>69.769</v>
       </c>
       <c r="I23" t="str">
         <v>Automatic</v>
@@ -1945,7 +2125,7 @@
         <v>Left</v>
       </c>
       <c r="K23" t="str">
-        <v>Unknown</v>
+        <v>Left</v>
       </c>
       <c r="L23">
         <v>0</v>
@@ -1974,19 +2154,31 @@
       <c r="T23">
         <v>0</v>
       </c>
+      <c r="U23" t="str">
+        <v/>
+      </c>
+      <c r="V23" t="str">
+        <v/>
+      </c>
       <c r="W23">
         <v>1</v>
       </c>
       <c r="X23" t="str">
-        <v>70/34</v>
+        <v>69/36</v>
       </c>
       <c r="Y23">
-        <v>900</v>
+        <v>300</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SE-7113</v>
+        <v>SE-7013</v>
+      </c>
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v/>
       </c>
       <c r="D24" t="str">
         <v>KYN-KJT</v>
@@ -1998,10 +2190,10 @@
         <v>DN</v>
       </c>
       <c r="G24" t="str">
-        <v>71/34</v>
+        <v>70/34</v>
       </c>
       <c r="H24">
-        <v>71.668</v>
+        <v>70.719</v>
       </c>
       <c r="I24" t="str">
         <v>Automatic</v>
@@ -2039,19 +2231,31 @@
       <c r="T24">
         <v>0</v>
       </c>
+      <c r="U24" t="str">
+        <v/>
+      </c>
+      <c r="V24" t="str">
+        <v/>
+      </c>
       <c r="W24">
         <v>1</v>
       </c>
       <c r="X24" t="str">
-        <v>71/34</v>
+        <v>70/34</v>
       </c>
       <c r="Y24">
-        <v>750</v>
+        <v>900</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SE-7223</v>
+        <v>SE-7113</v>
+      </c>
+      <c r="B25" t="str">
+        <v/>
+      </c>
+      <c r="C25" t="str">
+        <v/>
       </c>
       <c r="D25" t="str">
         <v>KYN-KJT</v>
@@ -2063,10 +2267,10 @@
         <v>DN</v>
       </c>
       <c r="G25" t="str">
-        <v>72/40</v>
+        <v>71/34</v>
       </c>
       <c r="H25">
-        <v>72.80199999999999</v>
+        <v>71.668</v>
       </c>
       <c r="I25" t="str">
         <v>Automatic</v>
@@ -2075,7 +2279,7 @@
         <v>Left</v>
       </c>
       <c r="K25" t="str">
-        <v>Left</v>
+        <v>Unknown</v>
       </c>
       <c r="L25">
         <v>0</v>
@@ -2104,19 +2308,31 @@
       <c r="T25">
         <v>0</v>
       </c>
+      <c r="U25" t="str">
+        <v/>
+      </c>
+      <c r="V25" t="str">
+        <v/>
+      </c>
       <c r="W25">
         <v>1</v>
       </c>
       <c r="X25" t="str">
-        <v>72/40</v>
+        <v>71/34</v>
       </c>
       <c r="Y25">
-        <v>350</v>
+        <v>750</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SE-7307</v>
+        <v>SE-7223</v>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
+        <v/>
       </c>
       <c r="D26" t="str">
         <v>KYN-KJT</v>
@@ -2128,10 +2344,10 @@
         <v>DN</v>
       </c>
       <c r="G26" t="str">
-        <v>73/16</v>
+        <v>72/40</v>
       </c>
       <c r="H26">
-        <v>73.292</v>
+        <v>72.80199999999999</v>
       </c>
       <c r="I26" t="str">
         <v>Automatic</v>
@@ -2140,7 +2356,7 @@
         <v>Left</v>
       </c>
       <c r="K26" t="str">
-        <v>Unknown</v>
+        <v>Left</v>
       </c>
       <c r="L26">
         <v>0</v>
@@ -2169,19 +2385,31 @@
       <c r="T26">
         <v>0</v>
       </c>
+      <c r="U26" t="str">
+        <v/>
+      </c>
+      <c r="V26" t="str">
+        <v/>
+      </c>
       <c r="W26">
         <v>1</v>
       </c>
       <c r="X26" t="str">
-        <v>73/16</v>
+        <v>72/40</v>
       </c>
       <c r="Y26">
-        <v>450</v>
+        <v>350</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SE-7403</v>
+        <v>SE-7307</v>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v/>
       </c>
       <c r="D27" t="str">
         <v>KYN-KJT</v>
@@ -2193,10 +2421,10 @@
         <v>DN</v>
       </c>
       <c r="G27" t="str">
-        <v>74/08</v>
+        <v>73/16</v>
       </c>
       <c r="H27">
-        <v>74.092</v>
+        <v>73.292</v>
       </c>
       <c r="I27" t="str">
         <v>Automatic</v>
@@ -2205,7 +2433,7 @@
         <v>Left</v>
       </c>
       <c r="K27" t="str">
-        <v>Left</v>
+        <v>Unknown</v>
       </c>
       <c r="L27">
         <v>0</v>
@@ -2234,19 +2462,31 @@
       <c r="T27">
         <v>0</v>
       </c>
+      <c r="U27" t="str">
+        <v/>
+      </c>
+      <c r="V27" t="str">
+        <v/>
+      </c>
       <c r="W27">
         <v>1</v>
       </c>
       <c r="X27" t="str">
-        <v>74/08</v>
+        <v>73/16</v>
       </c>
       <c r="Y27">
-        <v>500</v>
+        <v>450</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SE-7413</v>
+        <v>SE-7403</v>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v/>
       </c>
       <c r="D28" t="str">
         <v>KYN-KJT</v>
@@ -2258,10 +2498,10 @@
         <v>DN</v>
       </c>
       <c r="G28" t="str">
-        <v>74/42</v>
+        <v>74/08</v>
       </c>
       <c r="H28">
-        <v>74.797</v>
+        <v>74.092</v>
       </c>
       <c r="I28" t="str">
         <v>Automatic</v>
@@ -2270,7 +2510,7 @@
         <v>Left</v>
       </c>
       <c r="K28" t="str">
-        <v>Right</v>
+        <v>Left</v>
       </c>
       <c r="L28">
         <v>0</v>
@@ -2299,11 +2539,17 @@
       <c r="T28">
         <v>0</v>
       </c>
+      <c r="U28" t="str">
+        <v/>
+      </c>
+      <c r="V28" t="str">
+        <v/>
+      </c>
       <c r="W28">
         <v>1</v>
       </c>
       <c r="X28" t="str">
-        <v>74/42</v>
+        <v>74/08</v>
       </c>
       <c r="Y28">
         <v>500</v>
@@ -2311,7 +2557,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>SE-7507</v>
+        <v>SE-7413</v>
+      </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v/>
       </c>
       <c r="D29" t="str">
         <v>KYN-KJT</v>
@@ -2323,10 +2575,10 @@
         <v>DN</v>
       </c>
       <c r="G29" t="str">
-        <v>75/20</v>
+        <v>74/42</v>
       </c>
       <c r="H29">
-        <v>75.372</v>
+        <v>74.797</v>
       </c>
       <c r="I29" t="str">
         <v>Automatic</v>
@@ -2335,7 +2587,7 @@
         <v>Left</v>
       </c>
       <c r="K29" t="str">
-        <v>Unknown</v>
+        <v>Right</v>
       </c>
       <c r="L29">
         <v>0</v>
@@ -2364,19 +2616,31 @@
       <c r="T29">
         <v>0</v>
       </c>
+      <c r="U29" t="str">
+        <v/>
+      </c>
+      <c r="V29" t="str">
+        <v/>
+      </c>
       <c r="W29">
         <v>1</v>
       </c>
       <c r="X29" t="str">
-        <v>75/20</v>
+        <v>74/42</v>
       </c>
       <c r="Y29">
-        <v>600</v>
+        <v>500</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Gate-16</v>
+        <v>SE-7507</v>
+      </c>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
+        <v/>
       </c>
       <c r="D30" t="str">
         <v>KYN-KJT</v>
@@ -2388,19 +2652,19 @@
         <v>DN</v>
       </c>
       <c r="G30" t="str">
-        <v>75/46</v>
+        <v>75/20</v>
       </c>
       <c r="H30">
-        <v>75.937</v>
+        <v>75.372</v>
       </c>
       <c r="I30" t="str">
-        <v>Gate</v>
+        <v>Automatic</v>
       </c>
       <c r="J30" t="str">
         <v>Left</v>
       </c>
       <c r="K30" t="str">
-        <v>Left</v>
+        <v>Unknown</v>
       </c>
       <c r="L30">
         <v>0</v>
@@ -2429,19 +2693,31 @@
       <c r="T30">
         <v>0</v>
       </c>
+      <c r="U30" t="str">
+        <v/>
+      </c>
+      <c r="V30" t="str">
+        <v/>
+      </c>
       <c r="W30">
         <v>1</v>
       </c>
       <c r="X30" t="str">
-        <v>75/46</v>
+        <v>75/20</v>
       </c>
       <c r="Y30">
-        <v>350</v>
+        <v>600</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>SE-7613</v>
+        <v>Gate-16</v>
+      </c>
+      <c r="B31" t="str">
+        <v/>
+      </c>
+      <c r="C31" t="str">
+        <v/>
       </c>
       <c r="D31" t="str">
         <v>KYN-KJT</v>
@@ -2453,13 +2729,13 @@
         <v>DN</v>
       </c>
       <c r="G31" t="str">
-        <v>76/36</v>
+        <v>75/46</v>
       </c>
       <c r="H31">
-        <v>76.737</v>
+        <v>75.937</v>
       </c>
       <c r="I31" t="str">
-        <v>Automatic</v>
+        <v>Gate</v>
       </c>
       <c r="J31" t="str">
         <v>Left</v>
@@ -2494,25 +2770,31 @@
       <c r="T31">
         <v>0</v>
       </c>
+      <c r="U31" t="str">
+        <v/>
+      </c>
+      <c r="V31" t="str">
+        <v/>
+      </c>
       <c r="W31">
         <v>1</v>
       </c>
       <c r="X31" t="str">
-        <v>76/36</v>
+        <v>75/46</v>
       </c>
       <c r="Y31">
-        <v>250</v>
+        <v>350</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>VGI S-2</v>
+        <v>SE-7613</v>
       </c>
       <c r="B32" t="str">
-        <v>VGI</v>
+        <v/>
       </c>
       <c r="C32" t="str">
-        <v>Vangani</v>
+        <v/>
       </c>
       <c r="D32" t="str">
         <v>KYN-KJT</v>
@@ -2524,19 +2806,19 @@
         <v>DN</v>
       </c>
       <c r="G32" t="str">
-        <v>77/12</v>
+        <v>76/36</v>
       </c>
       <c r="H32">
-        <v>77.137</v>
+        <v>76.737</v>
       </c>
       <c r="I32" t="str">
-        <v>Manual</v>
+        <v>Automatic</v>
       </c>
       <c r="J32" t="str">
         <v>Left</v>
       </c>
       <c r="K32" t="str">
-        <v>Unknown</v>
+        <v>Left</v>
       </c>
       <c r="L32">
         <v>0</v>
@@ -2551,7 +2833,7 @@
         <v>0</v>
       </c>
       <c r="P32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q32">
         <v>0</v>
@@ -2565,19 +2847,25 @@
       <c r="T32">
         <v>0</v>
       </c>
+      <c r="U32" t="str">
+        <v/>
+      </c>
+      <c r="V32" t="str">
+        <v/>
+      </c>
       <c r="W32">
         <v>1</v>
       </c>
       <c r="X32" t="str">
-        <v>77/12</v>
+        <v>76/36</v>
       </c>
       <c r="Y32">
-        <v>300</v>
+        <v>250</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>VGI S-7</v>
+        <v>VGI S-2</v>
       </c>
       <c r="B33" t="str">
         <v>VGI</v>
@@ -2595,10 +2883,10 @@
         <v>DN</v>
       </c>
       <c r="G33" t="str">
-        <v>77/30</v>
+        <v>77/12</v>
       </c>
       <c r="H33">
-        <v>77.557</v>
+        <v>77.137</v>
       </c>
       <c r="I33" t="str">
         <v>Manual</v>
@@ -2622,39 +2910,39 @@
         <v>0</v>
       </c>
       <c r="P33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T33">
         <v>0</v>
       </c>
       <c r="U33" t="str">
-        <v>RI: L1=DN LL</v>
+        <v/>
       </c>
       <c r="V33" t="str">
-        <v>Book shows one left arm on top of vertical stem</v>
+        <v/>
       </c>
       <c r="W33">
         <v>1</v>
       </c>
       <c r="X33" t="str">
-        <v>77/30</v>
+        <v>77/12</v>
       </c>
       <c r="Y33">
-        <v>350</v>
+        <v>300</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>VGI S-3</v>
+        <v>VGI S-7</v>
       </c>
       <c r="B34" t="str">
         <v>VGI</v>
@@ -2672,19 +2960,19 @@
         <v>DN</v>
       </c>
       <c r="G34" t="str">
-        <v>PF-1 STR</v>
+        <v>77/30</v>
       </c>
       <c r="H34">
-        <v>78.516</v>
+        <v>77.557</v>
       </c>
       <c r="I34" t="str">
         <v>Manual</v>
       </c>
       <c r="J34" t="str">
-        <v>Extreme Left</v>
+        <v>Left</v>
       </c>
       <c r="K34" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="L34">
         <v>0</v>
@@ -2693,36 +2981,45 @@
         <v>0</v>
       </c>
       <c r="N34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P34">
         <v>0</v>
       </c>
       <c r="Q34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T34">
         <v>0</v>
       </c>
+      <c r="U34" t="str">
+        <v>RI: L1=DN LL</v>
+      </c>
+      <c r="V34" t="str">
+        <v>Book shows one left arm on top of vertical stem</v>
+      </c>
       <c r="W34">
         <v>1</v>
       </c>
+      <c r="X34" t="str">
+        <v>77/30</v>
+      </c>
       <c r="Y34">
-        <v>300</v>
+        <v>350</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>VGI S-8</v>
+        <v>VGI S-3</v>
       </c>
       <c r="B35" t="str">
         <v>VGI</v>
@@ -2740,19 +3037,19 @@
         <v>DN</v>
       </c>
       <c r="G35" t="str">
-        <v>78/48</v>
+        <v>PF-1 STR</v>
       </c>
       <c r="H35">
-        <v>78.891</v>
+        <v>78.516</v>
       </c>
       <c r="I35" t="str">
         <v>Manual</v>
       </c>
       <c r="J35" t="str">
-        <v>Left</v>
+        <v>Extreme Left</v>
       </c>
       <c r="K35" t="str">
-        <v>Unknown</v>
+        <v>Right</v>
       </c>
       <c r="L35">
         <v>0</v>
@@ -2761,10 +3058,10 @@
         <v>0</v>
       </c>
       <c r="N35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P35">
         <v>0</v>
@@ -2781,11 +3078,17 @@
       <c r="T35">
         <v>0</v>
       </c>
+      <c r="U35" t="str">
+        <v/>
+      </c>
+      <c r="V35" t="str">
+        <v/>
+      </c>
       <c r="W35">
         <v>1</v>
       </c>
       <c r="X35" t="str">
-        <v>78/48</v>
+        <v/>
       </c>
       <c r="Y35">
         <v>300</v>
@@ -2793,7 +3096,13 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Gate-18</v>
+        <v>VGI S-8</v>
+      </c>
+      <c r="B36" t="str">
+        <v>VGI</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Vangani</v>
       </c>
       <c r="D36" t="str">
         <v>KYN-KJT</v>
@@ -2805,19 +3114,19 @@
         <v>DN</v>
       </c>
       <c r="G36" t="str">
-        <v>79/38</v>
+        <v>78/48</v>
       </c>
       <c r="H36">
-        <v>79.711</v>
+        <v>78.891</v>
       </c>
       <c r="I36" t="str">
-        <v>Gate</v>
+        <v>Manual</v>
       </c>
       <c r="J36" t="str">
         <v>Left</v>
       </c>
       <c r="K36" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="L36">
         <v>0</v>
@@ -2846,11 +3155,17 @@
       <c r="T36">
         <v>0</v>
       </c>
+      <c r="U36" t="str">
+        <v/>
+      </c>
+      <c r="V36" t="str">
+        <v/>
+      </c>
       <c r="W36">
         <v>1</v>
       </c>
       <c r="X36" t="str">
-        <v>79/38</v>
+        <v>78/48</v>
       </c>
       <c r="Y36">
         <v>300</v>
@@ -2858,7 +3173,13 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>SE-8009</v>
+        <v>Gate-18</v>
+      </c>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v/>
       </c>
       <c r="D37" t="str">
         <v>KYN-KJT</v>
@@ -2870,19 +3191,19 @@
         <v>DN</v>
       </c>
       <c r="G37" t="str">
-        <v>80/20</v>
+        <v>79/38</v>
       </c>
       <c r="H37">
-        <v>80.417</v>
+        <v>79.711</v>
       </c>
       <c r="I37" t="str">
-        <v>Automatic</v>
+        <v>Gate</v>
       </c>
       <c r="J37" t="str">
         <v>Left</v>
       </c>
       <c r="K37" t="str">
-        <v>Unknown</v>
+        <v>Right</v>
       </c>
       <c r="L37">
         <v>0</v>
@@ -2911,11 +3232,17 @@
       <c r="T37">
         <v>0</v>
       </c>
+      <c r="U37" t="str">
+        <v/>
+      </c>
+      <c r="V37" t="str">
+        <v/>
+      </c>
       <c r="W37">
         <v>1</v>
       </c>
       <c r="X37" t="str">
-        <v>80/20</v>
+        <v>79/38</v>
       </c>
       <c r="Y37">
         <v>300</v>
@@ -2923,7 +3250,13 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Gate-19</v>
+        <v>SE-8009</v>
+      </c>
+      <c r="B38" t="str">
+        <v/>
+      </c>
+      <c r="C38" t="str">
+        <v/>
       </c>
       <c r="D38" t="str">
         <v>KYN-KJT</v>
@@ -2935,13 +3268,13 @@
         <v>DN</v>
       </c>
       <c r="G38" t="str">
-        <v>81/08</v>
+        <v>80/20</v>
       </c>
       <c r="H38">
-        <v>81.114</v>
+        <v>80.417</v>
       </c>
       <c r="I38" t="str">
-        <v>Gate</v>
+        <v>Automatic</v>
       </c>
       <c r="J38" t="str">
         <v>Left</v>
@@ -2976,19 +3309,31 @@
       <c r="T38">
         <v>0</v>
       </c>
+      <c r="U38" t="str">
+        <v/>
+      </c>
+      <c r="V38" t="str">
+        <v/>
+      </c>
       <c r="W38">
         <v>1</v>
       </c>
       <c r="X38" t="str">
-        <v>81/08</v>
+        <v>80/20</v>
       </c>
       <c r="Y38">
-        <v>500</v>
+        <v>300</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>SE-8115</v>
+        <v>Gate-19</v>
+      </c>
+      <c r="B39" t="str">
+        <v/>
+      </c>
+      <c r="C39" t="str">
+        <v/>
       </c>
       <c r="D39" t="str">
         <v>KYN-KJT</v>
@@ -3000,13 +3345,13 @@
         <v>DN</v>
       </c>
       <c r="G39" t="str">
-        <v>81/34</v>
+        <v>81/08</v>
       </c>
       <c r="H39">
-        <v>81.73400000000001</v>
+        <v>81.114</v>
       </c>
       <c r="I39" t="str">
-        <v>Automatic</v>
+        <v>Gate</v>
       </c>
       <c r="J39" t="str">
         <v>Left</v>
@@ -3041,19 +3386,31 @@
       <c r="T39">
         <v>0</v>
       </c>
+      <c r="U39" t="str">
+        <v/>
+      </c>
+      <c r="V39" t="str">
+        <v/>
+      </c>
       <c r="W39">
         <v>1</v>
       </c>
       <c r="X39" t="str">
-        <v>81/34</v>
+        <v>81/08</v>
       </c>
       <c r="Y39">
-        <v>450</v>
+        <v>500</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>SE-8205</v>
+        <v>SE-8115</v>
+      </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v/>
       </c>
       <c r="D40" t="str">
         <v>KYN-KJT</v>
@@ -3065,10 +3422,10 @@
         <v>DN</v>
       </c>
       <c r="G40" t="str">
-        <v>82/14</v>
+        <v>81/34</v>
       </c>
       <c r="H40">
-        <v>82.275</v>
+        <v>81.73400000000001</v>
       </c>
       <c r="I40" t="str">
         <v>Automatic</v>
@@ -3077,7 +3434,7 @@
         <v>Left</v>
       </c>
       <c r="K40" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="L40">
         <v>0</v>
@@ -3106,19 +3463,31 @@
       <c r="T40">
         <v>0</v>
       </c>
+      <c r="U40" t="str">
+        <v/>
+      </c>
+      <c r="V40" t="str">
+        <v/>
+      </c>
       <c r="W40">
         <v>1</v>
       </c>
       <c r="X40" t="str">
-        <v>82/14</v>
+        <v>81/34</v>
       </c>
       <c r="Y40">
-        <v>400</v>
+        <v>450</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>SE-8303</v>
+        <v>SE-8205</v>
+      </c>
+      <c r="B41" t="str">
+        <v/>
+      </c>
+      <c r="C41" t="str">
+        <v/>
       </c>
       <c r="D41" t="str">
         <v>KYN-KJT</v>
@@ -3130,10 +3499,10 @@
         <v>DN</v>
       </c>
       <c r="G41" t="str">
-        <v>83/08</v>
+        <v>82/14</v>
       </c>
       <c r="H41">
-        <v>82.97</v>
+        <v>82.275</v>
       </c>
       <c r="I41" t="str">
         <v>Automatic</v>
@@ -3142,7 +3511,7 @@
         <v>Left</v>
       </c>
       <c r="K41" t="str">
-        <v>Unknown</v>
+        <v>Right</v>
       </c>
       <c r="L41">
         <v>0</v>
@@ -3171,19 +3540,31 @@
       <c r="T41">
         <v>0</v>
       </c>
+      <c r="U41" t="str">
+        <v/>
+      </c>
+      <c r="V41" t="str">
+        <v/>
+      </c>
       <c r="W41">
         <v>1</v>
       </c>
       <c r="X41" t="str">
-        <v>83/08</v>
+        <v>82/14</v>
       </c>
       <c r="Y41">
-        <v>600</v>
+        <v>400</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Gate- 20</v>
+        <v>SE-8303</v>
+      </c>
+      <c r="B42" t="str">
+        <v/>
+      </c>
+      <c r="C42" t="str">
+        <v/>
       </c>
       <c r="D42" t="str">
         <v>KYN-KJT</v>
@@ -3195,10 +3576,10 @@
         <v>DN</v>
       </c>
       <c r="G42" t="str">
-        <v>83/40</v>
+        <v>83/08</v>
       </c>
       <c r="H42">
-        <v>83.795</v>
+        <v>82.97</v>
       </c>
       <c r="I42" t="str">
         <v>Automatic</v>
@@ -3207,7 +3588,7 @@
         <v>Left</v>
       </c>
       <c r="K42" t="str">
-        <v>Left</v>
+        <v>Unknown</v>
       </c>
       <c r="L42">
         <v>0</v>
@@ -3236,25 +3617,31 @@
       <c r="T42">
         <v>0</v>
       </c>
+      <c r="U42" t="str">
+        <v/>
+      </c>
+      <c r="V42" t="str">
+        <v/>
+      </c>
       <c r="W42">
         <v>1</v>
       </c>
       <c r="X42" t="str">
-        <v>83/40</v>
+        <v>83/08</v>
       </c>
       <c r="Y42">
-        <v>700</v>
+        <v>600</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>NRL S-27</v>
+        <v>Gate- 20</v>
       </c>
       <c r="B43" t="str">
-        <v>NRL</v>
+        <v/>
       </c>
       <c r="C43" t="str">
-        <v>Neral</v>
+        <v/>
       </c>
       <c r="D43" t="str">
         <v>KYN-KJT</v>
@@ -3266,19 +3653,19 @@
         <v>DN</v>
       </c>
       <c r="G43" t="str">
-        <v>84/26</v>
+        <v>83/40</v>
       </c>
       <c r="H43">
-        <v>84.561</v>
+        <v>83.795</v>
       </c>
       <c r="I43" t="str">
-        <v>Manual</v>
+        <v>Automatic</v>
       </c>
       <c r="J43" t="str">
         <v>Left</v>
       </c>
       <c r="K43" t="str">
-        <v>Unknown</v>
+        <v>Left</v>
       </c>
       <c r="L43">
         <v>0</v>
@@ -3296,36 +3683,36 @@
         <v>0</v>
       </c>
       <c r="Q43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R43">
         <v>0</v>
       </c>
       <c r="S43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U43" t="str">
-        <v>RI: L1=DN LL; R1=UDL</v>
+        <v/>
       </c>
       <c r="V43" t="str">
-        <v>Book shows one left and one right arm on top of vertical stem</v>
+        <v/>
       </c>
       <c r="W43">
         <v>1</v>
       </c>
       <c r="X43" t="str">
-        <v>84/26</v>
+        <v>83/40</v>
       </c>
       <c r="Y43">
-        <v>600</v>
+        <v>700</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>NRL S-21</v>
+        <v>NRL S-27</v>
       </c>
       <c r="B44" t="str">
         <v>NRL</v>
@@ -3343,16 +3730,16 @@
         <v>DN</v>
       </c>
       <c r="G44" t="str">
-        <v>85/40</v>
+        <v>84/26</v>
       </c>
       <c r="H44">
-        <v>85.666</v>
+        <v>84.561</v>
       </c>
       <c r="I44" t="str">
         <v>Manual</v>
       </c>
       <c r="J44" t="str">
-        <v>Extreme Left</v>
+        <v>Left</v>
       </c>
       <c r="K44" t="str">
         <v>Unknown</v>
@@ -3364,39 +3751,45 @@
         <v>0</v>
       </c>
       <c r="N44">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P44">
         <v>0</v>
       </c>
       <c r="Q44">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R44">
         <v>0</v>
       </c>
       <c r="S44">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T44">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="U44" t="str">
+        <v>RI: L1=DN LL; R1=UDL</v>
+      </c>
+      <c r="V44" t="str">
+        <v>Book shows one left and one right arm on top of vertical stem</v>
       </c>
       <c r="W44">
         <v>1</v>
       </c>
       <c r="X44" t="str">
-        <v>85/40</v>
+        <v>84/26</v>
       </c>
       <c r="Y44">
-        <v>950</v>
+        <v>600</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>NRL S-18</v>
+        <v>NRL S-21</v>
       </c>
       <c r="B45" t="str">
         <v>NRL</v>
@@ -3414,16 +3807,16 @@
         <v>DN</v>
       </c>
       <c r="G45" t="str">
-        <v>PF-1 STR</v>
+        <v>85/40</v>
       </c>
       <c r="H45">
-        <v>86.24000000000001</v>
+        <v>85.666</v>
       </c>
       <c r="I45" t="str">
         <v>Manual</v>
       </c>
       <c r="J45" t="str">
-        <v>Left</v>
+        <v>Extreme Left</v>
       </c>
       <c r="K45" t="str">
         <v>Unknown</v>
@@ -3435,16 +3828,16 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P45">
         <v>0</v>
       </c>
       <c r="Q45">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R45">
         <v>0</v>
@@ -3455,16 +3848,25 @@
       <c r="T45">
         <v>0</v>
       </c>
+      <c r="U45" t="str">
+        <v/>
+      </c>
+      <c r="V45" t="str">
+        <v/>
+      </c>
       <c r="W45">
         <v>1</v>
       </c>
+      <c r="X45" t="str">
+        <v>85/40</v>
+      </c>
       <c r="Y45">
-        <v>600</v>
+        <v>950</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>NRL S-17</v>
+        <v>NRL S-18</v>
       </c>
       <c r="B46" t="str">
         <v>NRL</v>
@@ -3482,10 +3884,10 @@
         <v>DN</v>
       </c>
       <c r="G46" t="str">
-        <v>87/06</v>
+        <v>PF-1 STR</v>
       </c>
       <c r="H46">
-        <v>87.03999999999999</v>
+        <v>86.24000000000001</v>
       </c>
       <c r="I46" t="str">
         <v>Manual</v>
@@ -3494,7 +3896,7 @@
         <v>Left</v>
       </c>
       <c r="K46" t="str">
-        <v>Left</v>
+        <v>Unknown</v>
       </c>
       <c r="L46">
         <v>0</v>
@@ -3512,7 +3914,7 @@
         <v>0</v>
       </c>
       <c r="Q46">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R46">
         <v>0</v>
@@ -3523,19 +3925,31 @@
       <c r="T46">
         <v>0</v>
       </c>
+      <c r="U46" t="str">
+        <v/>
+      </c>
+      <c r="V46" t="str">
+        <v/>
+      </c>
       <c r="W46">
         <v>1</v>
       </c>
       <c r="X46" t="str">
-        <v>87/06</v>
+        <v/>
       </c>
       <c r="Y46">
-        <v>250</v>
+        <v>600</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>SE-8801</v>
+        <v>NRL S-17</v>
+      </c>
+      <c r="B47" t="str">
+        <v>NRL</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Neral</v>
       </c>
       <c r="D47" t="str">
         <v>KYN-KJT</v>
@@ -3547,19 +3961,19 @@
         <v>DN</v>
       </c>
       <c r="G47" t="str">
-        <v>87/46</v>
+        <v>87/06</v>
       </c>
       <c r="H47">
-        <v>87.84</v>
+        <v>87.03999999999999</v>
       </c>
       <c r="I47" t="str">
-        <v>Automatic</v>
+        <v>Manual</v>
       </c>
       <c r="J47" t="str">
         <v>Left</v>
       </c>
       <c r="K47" t="str">
-        <v>Right</v>
+        <v>Left</v>
       </c>
       <c r="L47">
         <v>0</v>
@@ -3588,19 +4002,31 @@
       <c r="T47">
         <v>0</v>
       </c>
+      <c r="U47" t="str">
+        <v/>
+      </c>
+      <c r="V47" t="str">
+        <v/>
+      </c>
       <c r="W47">
         <v>1</v>
       </c>
       <c r="X47" t="str">
-        <v>87/46</v>
+        <v>87/06</v>
       </c>
       <c r="Y47">
-        <v>300</v>
+        <v>250</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>SE-8813</v>
+        <v>SE-8801</v>
+      </c>
+      <c r="B48" t="str">
+        <v/>
+      </c>
+      <c r="C48" t="str">
+        <v/>
       </c>
       <c r="D48" t="str">
         <v>KYN-KJT</v>
@@ -3612,10 +4038,10 @@
         <v>DN</v>
       </c>
       <c r="G48" t="str">
-        <v>88/32</v>
+        <v>87/46</v>
       </c>
       <c r="H48">
-        <v>88.64</v>
+        <v>87.84</v>
       </c>
       <c r="I48" t="str">
         <v>Automatic</v>
@@ -3624,7 +4050,7 @@
         <v>Left</v>
       </c>
       <c r="K48" t="str">
-        <v>Unknown</v>
+        <v>Right</v>
       </c>
       <c r="L48">
         <v>0</v>
@@ -3653,19 +4079,31 @@
       <c r="T48">
         <v>0</v>
       </c>
+      <c r="U48" t="str">
+        <v/>
+      </c>
+      <c r="V48" t="str">
+        <v/>
+      </c>
       <c r="W48">
         <v>1</v>
       </c>
       <c r="X48" t="str">
-        <v>88/32</v>
+        <v>87/46</v>
       </c>
       <c r="Y48">
-        <v>700</v>
+        <v>300</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Gate-22</v>
+        <v>SE-8813</v>
+      </c>
+      <c r="B49" t="str">
+        <v/>
+      </c>
+      <c r="C49" t="str">
+        <v/>
       </c>
       <c r="D49" t="str">
         <v>KYN-KJT</v>
@@ -3677,13 +4115,13 @@
         <v>DN</v>
       </c>
       <c r="G49" t="str">
-        <v>89/24</v>
+        <v>88/32</v>
       </c>
       <c r="H49">
-        <v>89.48</v>
+        <v>88.64</v>
       </c>
       <c r="I49" t="str">
-        <v>Gate</v>
+        <v>Automatic</v>
       </c>
       <c r="J49" t="str">
         <v>Left</v>
@@ -3718,19 +4156,31 @@
       <c r="T49">
         <v>0</v>
       </c>
+      <c r="U49" t="str">
+        <v/>
+      </c>
+      <c r="V49" t="str">
+        <v/>
+      </c>
       <c r="W49">
         <v>1</v>
       </c>
       <c r="X49" t="str">
-        <v>89/24</v>
+        <v>88/32</v>
       </c>
       <c r="Y49">
-        <v>600</v>
+        <v>700</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>SE-9007</v>
+        <v>Gate-22</v>
+      </c>
+      <c r="B50" t="str">
+        <v/>
+      </c>
+      <c r="C50" t="str">
+        <v/>
       </c>
       <c r="D50" t="str">
         <v>KYN-KJT</v>
@@ -3742,13 +4192,13 @@
         <v>DN</v>
       </c>
       <c r="G50" t="str">
-        <v>90/18</v>
+        <v>89/24</v>
       </c>
       <c r="H50">
-        <v>90.28</v>
+        <v>89.48</v>
       </c>
       <c r="I50" t="str">
-        <v>Automatic</v>
+        <v>Gate</v>
       </c>
       <c r="J50" t="str">
         <v>Left</v>
@@ -3783,19 +4233,31 @@
       <c r="T50">
         <v>0</v>
       </c>
+      <c r="U50" t="str">
+        <v/>
+      </c>
+      <c r="V50" t="str">
+        <v/>
+      </c>
       <c r="W50">
         <v>1</v>
       </c>
       <c r="X50" t="str">
-        <v>90/18</v>
+        <v>89/24</v>
       </c>
       <c r="Y50">
-        <v>800</v>
+        <v>600</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>SE-9105</v>
+        <v>SE-9007</v>
+      </c>
+      <c r="B51" t="str">
+        <v/>
+      </c>
+      <c r="C51" t="str">
+        <v/>
       </c>
       <c r="D51" t="str">
         <v>KYN-KJT</v>
@@ -3807,10 +4269,10 @@
         <v>DN</v>
       </c>
       <c r="G51" t="str">
-        <v>91/10</v>
+        <v>90/18</v>
       </c>
       <c r="H51">
-        <v>91.14</v>
+        <v>90.28</v>
       </c>
       <c r="I51" t="str">
         <v>Automatic</v>
@@ -3848,25 +4310,31 @@
       <c r="T51">
         <v>0</v>
       </c>
+      <c r="U51" t="str">
+        <v/>
+      </c>
+      <c r="V51" t="str">
+        <v/>
+      </c>
       <c r="W51">
         <v>1</v>
       </c>
       <c r="X51" t="str">
-        <v>91/10</v>
+        <v>90/18</v>
       </c>
       <c r="Y51">
-        <v>1200</v>
+        <v>800</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>BVS S-2</v>
+        <v>SE-9105</v>
       </c>
       <c r="B52" t="str">
-        <v>BVS</v>
+        <v/>
       </c>
       <c r="C52" t="str">
-        <v>Bhivpuri</v>
+        <v/>
       </c>
       <c r="D52" t="str">
         <v>KYN-KJT</v>
@@ -3878,13 +4346,13 @@
         <v>DN</v>
       </c>
       <c r="G52" t="str">
-        <v>92/06</v>
+        <v>91/10</v>
       </c>
       <c r="H52">
-        <v>92.03</v>
+        <v>91.14</v>
       </c>
       <c r="I52" t="str">
-        <v>Manual</v>
+        <v>Automatic</v>
       </c>
       <c r="J52" t="str">
         <v>Left</v>
@@ -3908,36 +4376,36 @@
         <v>0</v>
       </c>
       <c r="Q52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R52">
         <v>0</v>
       </c>
       <c r="S52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T52">
         <v>0</v>
       </c>
       <c r="U52" t="str">
-        <v>RI: L1=DN LL</v>
+        <v/>
       </c>
       <c r="V52" t="str">
-        <v>Book shows one left arm on top of vertical stem</v>
+        <v/>
       </c>
       <c r="W52">
         <v>1</v>
       </c>
       <c r="X52" t="str">
-        <v>92/06</v>
+        <v>91/10</v>
       </c>
       <c r="Y52">
-        <v>1000</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>BVS S-3</v>
+        <v>BVS S-2</v>
       </c>
       <c r="B53" t="str">
         <v>BVS</v>
@@ -3955,16 +4423,16 @@
         <v>DN</v>
       </c>
       <c r="G53" t="str">
-        <v>93/16</v>
+        <v>92/06</v>
       </c>
       <c r="H53">
-        <v>93.18299999999999</v>
+        <v>92.03</v>
       </c>
       <c r="I53" t="str">
         <v>Manual</v>
       </c>
       <c r="J53" t="str">
-        <v>Gantry</v>
+        <v>Left</v>
       </c>
       <c r="K53" t="str">
         <v>Unknown</v>
@@ -3985,27 +4453,36 @@
         <v>0</v>
       </c>
       <c r="Q53">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R53">
         <v>0</v>
       </c>
       <c r="S53">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T53">
         <v>0</v>
       </c>
+      <c r="U53" t="str">
+        <v>RI: L1=DN LL</v>
+      </c>
+      <c r="V53" t="str">
+        <v>Book shows one left arm on top of vertical stem</v>
+      </c>
       <c r="W53">
         <v>1</v>
       </c>
+      <c r="X53" t="str">
+        <v>92/06</v>
+      </c>
       <c r="Y53">
-        <v>500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>BVS S-8</v>
+        <v>BVS S-3</v>
       </c>
       <c r="B54" t="str">
         <v>BVS</v>
@@ -4023,16 +4500,16 @@
         <v>DN</v>
       </c>
       <c r="G54" t="str">
-        <v>94/06</v>
+        <v>93/16</v>
       </c>
       <c r="H54">
-        <v>94.07300000000001</v>
+        <v>93.18299999999999</v>
       </c>
       <c r="I54" t="str">
         <v>Manual</v>
       </c>
       <c r="J54" t="str">
-        <v>Left</v>
+        <v>Gantry</v>
       </c>
       <c r="K54" t="str">
         <v>Unknown</v>
@@ -4064,16 +4541,31 @@
       <c r="T54">
         <v>0</v>
       </c>
+      <c r="U54" t="str">
+        <v/>
+      </c>
+      <c r="V54" t="str">
+        <v/>
+      </c>
       <c r="W54">
         <v>1</v>
       </c>
+      <c r="X54" t="str">
+        <v/>
+      </c>
       <c r="Y54">
-        <v>1000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Gate-25</v>
+        <v>BVS S-8</v>
+      </c>
+      <c r="B55" t="str">
+        <v>BVS</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Bhivpuri</v>
       </c>
       <c r="D55" t="str">
         <v>KYN-KJT</v>
@@ -4085,19 +4577,19 @@
         <v>DN</v>
       </c>
       <c r="G55" t="str">
-        <v>95/02</v>
+        <v>94/06</v>
       </c>
       <c r="H55">
-        <v>94.97800000000001</v>
+        <v>94.07300000000001</v>
       </c>
       <c r="I55" t="str">
-        <v>Gate</v>
+        <v>Manual</v>
       </c>
       <c r="J55" t="str">
         <v>Left</v>
       </c>
       <c r="K55" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="L55">
         <v>0</v>
@@ -4126,16 +4618,31 @@
       <c r="T55">
         <v>0</v>
       </c>
+      <c r="U55" t="str">
+        <v/>
+      </c>
+      <c r="V55" t="str">
+        <v/>
+      </c>
       <c r="W55">
         <v>1</v>
       </c>
+      <c r="X55" t="str">
+        <v/>
+      </c>
       <c r="Y55">
-        <v>600</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>SE-9511</v>
+        <v>Gate-25</v>
+      </c>
+      <c r="B56" t="str">
+        <v/>
+      </c>
+      <c r="C56" t="str">
+        <v/>
       </c>
       <c r="D56" t="str">
         <v>KYN-KJT</v>
@@ -4147,19 +4654,19 @@
         <v>DN</v>
       </c>
       <c r="G56" t="str">
-        <v>95/30</v>
+        <v>95/02</v>
       </c>
       <c r="H56">
-        <v>95.568</v>
+        <v>94.97800000000001</v>
       </c>
       <c r="I56" t="str">
-        <v>Automatic</v>
+        <v>Gate</v>
       </c>
       <c r="J56" t="str">
         <v>Left</v>
       </c>
       <c r="K56" t="str">
-        <v>Unknown</v>
+        <v>Right</v>
       </c>
       <c r="L56">
         <v>0</v>
@@ -4188,16 +4695,31 @@
       <c r="T56">
         <v>0</v>
       </c>
+      <c r="U56" t="str">
+        <v/>
+      </c>
+      <c r="V56" t="str">
+        <v/>
+      </c>
       <c r="W56">
         <v>1</v>
       </c>
+      <c r="X56" t="str">
+        <v/>
+      </c>
       <c r="Y56">
-        <v>500</v>
+        <v>600</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Gate-26</v>
+        <v>SE-9511</v>
+      </c>
+      <c r="B57" t="str">
+        <v/>
+      </c>
+      <c r="C57" t="str">
+        <v/>
       </c>
       <c r="D57" t="str">
         <v>KYN-KJT</v>
@@ -4209,13 +4731,13 @@
         <v>DN</v>
       </c>
       <c r="G57" t="str">
-        <v>96/10</v>
+        <v>95/30</v>
       </c>
       <c r="H57">
-        <v>96.158</v>
+        <v>95.568</v>
       </c>
       <c r="I57" t="str">
-        <v>Gate</v>
+        <v>Automatic</v>
       </c>
       <c r="J57" t="str">
         <v>Left</v>
@@ -4250,16 +4772,31 @@
       <c r="T57">
         <v>0</v>
       </c>
+      <c r="U57" t="str">
+        <v/>
+      </c>
+      <c r="V57" t="str">
+        <v/>
+      </c>
       <c r="W57">
         <v>1</v>
       </c>
+      <c r="X57" t="str">
+        <v/>
+      </c>
       <c r="Y57">
-        <v>900</v>
+        <v>500</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>SE-9615</v>
+        <v>Gate-26</v>
+      </c>
+      <c r="B58" t="str">
+        <v/>
+      </c>
+      <c r="C58" t="str">
+        <v/>
       </c>
       <c r="D58" t="str">
         <v>KYN-KJT</v>
@@ -4271,13 +4808,13 @@
         <v>DN</v>
       </c>
       <c r="G58" t="str">
-        <v>96/40</v>
+        <v>96/10</v>
       </c>
       <c r="H58">
-        <v>96.882</v>
+        <v>96.158</v>
       </c>
       <c r="I58" t="str">
-        <v>Automatic</v>
+        <v>Gate</v>
       </c>
       <c r="J58" t="str">
         <v>Left</v>
@@ -4312,16 +4849,31 @@
       <c r="T58">
         <v>0</v>
       </c>
+      <c r="U58" t="str">
+        <v/>
+      </c>
+      <c r="V58" t="str">
+        <v/>
+      </c>
       <c r="W58">
         <v>1</v>
       </c>
+      <c r="X58" t="str">
+        <v/>
+      </c>
       <c r="Y58">
-        <v>1200</v>
+        <v>900</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Gate-27</v>
+        <v>SE-9615</v>
+      </c>
+      <c r="B59" t="str">
+        <v/>
+      </c>
+      <c r="C59" t="str">
+        <v/>
       </c>
       <c r="D59" t="str">
         <v>KYN-KJT</v>
@@ -4333,10 +4885,10 @@
         <v>DN</v>
       </c>
       <c r="G59" t="str">
-        <v>97/30</v>
+        <v>96/40</v>
       </c>
       <c r="H59">
-        <v>97.604</v>
+        <v>96.882</v>
       </c>
       <c r="I59" t="str">
         <v>Automatic</v>
@@ -4374,16 +4926,31 @@
       <c r="T59">
         <v>0</v>
       </c>
+      <c r="U59" t="str">
+        <v/>
+      </c>
+      <c r="V59" t="str">
+        <v/>
+      </c>
       <c r="W59">
         <v>1</v>
       </c>
+      <c r="X59" t="str">
+        <v/>
+      </c>
       <c r="Y59">
-        <v>1400</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>SE-9803</v>
+        <v>Gate-27</v>
+      </c>
+      <c r="B60" t="str">
+        <v/>
+      </c>
+      <c r="C60" t="str">
+        <v/>
       </c>
       <c r="D60" t="str">
         <v>KYN-KJT</v>
@@ -4395,10 +4962,10 @@
         <v>DN</v>
       </c>
       <c r="G60" t="str">
-        <v>98/08</v>
+        <v>97/30</v>
       </c>
       <c r="H60">
-        <v>98.11699999999999</v>
+        <v>97.604</v>
       </c>
       <c r="I60" t="str">
         <v>Automatic</v>
@@ -4407,7 +4974,7 @@
         <v>Left</v>
       </c>
       <c r="K60" t="str">
-        <v>Right</v>
+        <v>Unknown</v>
       </c>
       <c r="L60">
         <v>0</v>
@@ -4436,90 +5003,179 @@
       <c r="T60">
         <v>0</v>
       </c>
+      <c r="U60" t="str">
+        <v/>
+      </c>
+      <c r="V60" t="str">
+        <v/>
+      </c>
       <c r="W60">
         <v>1</v>
       </c>
+      <c r="X60" t="str">
+        <v/>
+      </c>
       <c r="Y60">
-        <v>500</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
+        <v>SE-9803</v>
+      </c>
+      <c r="B61" t="str">
+        <v/>
+      </c>
+      <c r="C61" t="str">
+        <v/>
+      </c>
+      <c r="D61" t="str">
+        <v>KYN-KJT</v>
+      </c>
+      <c r="E61" t="str">
+        <v>DN SE</v>
+      </c>
+      <c r="F61" t="str">
+        <v>DN</v>
+      </c>
+      <c r="G61" t="str">
+        <v>98/08</v>
+      </c>
+      <c r="H61">
+        <v>98.11699999999999</v>
+      </c>
+      <c r="I61" t="str">
+        <v>Automatic</v>
+      </c>
+      <c r="J61" t="str">
+        <v>Left</v>
+      </c>
+      <c r="K61" t="str">
+        <v>Right</v>
+      </c>
+      <c r="L61">
+        <v>0</v>
+      </c>
+      <c r="M61">
+        <v>0</v>
+      </c>
+      <c r="N61">
+        <v>1</v>
+      </c>
+      <c r="O61">
+        <v>0</v>
+      </c>
+      <c r="P61">
+        <v>0</v>
+      </c>
+      <c r="Q61">
+        <v>0</v>
+      </c>
+      <c r="R61">
+        <v>0</v>
+      </c>
+      <c r="S61">
+        <v>0</v>
+      </c>
+      <c r="T61">
+        <v>0</v>
+      </c>
+      <c r="U61" t="str">
+        <v/>
+      </c>
+      <c r="V61" t="str">
+        <v/>
+      </c>
+      <c r="W61">
+        <v>1</v>
+      </c>
+      <c r="X61" t="str">
+        <v/>
+      </c>
+      <c r="Y61">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
         <v>KJT S-2</v>
       </c>
-      <c r="B61" t="str">
+      <c r="B62" t="str">
         <v>KJT</v>
       </c>
-      <c r="C61" t="str">
+      <c r="C62" t="str">
         <v>Karjat</v>
       </c>
-      <c r="D61" t="str">
-        <v>KYN-KJT</v>
-      </c>
-      <c r="E61" t="str">
-        <v>DN SE</v>
-      </c>
-      <c r="F61" t="str">
-        <v>DN</v>
-      </c>
-      <c r="G61" t="str">
+      <c r="D62" t="str">
+        <v>KYN-KJT</v>
+      </c>
+      <c r="E62" t="str">
+        <v>DN SE</v>
+      </c>
+      <c r="F62" t="str">
+        <v>DN</v>
+      </c>
+      <c r="G62" t="str">
         <v>98/30</v>
       </c>
-      <c r="H61">
+      <c r="H62">
         <v>98.632</v>
       </c>
-      <c r="I61" t="str">
+      <c r="I62" t="str">
         <v>Manual</v>
       </c>
-      <c r="J61" t="str">
-        <v>Left</v>
-      </c>
-      <c r="K61" t="str">
+      <c r="J62" t="str">
+        <v>Left</v>
+      </c>
+      <c r="K62" t="str">
         <v>Unknown</v>
       </c>
-      <c r="L61">
-        <v>0</v>
-      </c>
-      <c r="M61">
-        <v>0</v>
-      </c>
-      <c r="N61">
-        <v>1</v>
-      </c>
-      <c r="O61">
-        <v>0</v>
-      </c>
-      <c r="P61">
-        <v>0</v>
-      </c>
-      <c r="Q61">
-        <v>1</v>
-      </c>
-      <c r="R61">
-        <v>0</v>
-      </c>
-      <c r="S61">
-        <v>0</v>
-      </c>
-      <c r="T61">
+      <c r="L62">
+        <v>0</v>
+      </c>
+      <c r="M62">
+        <v>0</v>
+      </c>
+      <c r="N62">
+        <v>1</v>
+      </c>
+      <c r="O62">
+        <v>0</v>
+      </c>
+      <c r="P62">
+        <v>0</v>
+      </c>
+      <c r="Q62">
+        <v>1</v>
+      </c>
+      <c r="R62">
+        <v>0</v>
+      </c>
+      <c r="S62">
+        <v>0</v>
+      </c>
+      <c r="T62">
         <v>3</v>
       </c>
-      <c r="U61" t="str">
+      <c r="U62" t="str">
         <v>RI: R1= S-14; R2=EMU PF; R3= PF-3</v>
       </c>
-      <c r="V61" t="str">
+      <c r="V62" t="str">
         <v>Book shows three right arm on top of vertical stem</v>
       </c>
-      <c r="W61">
-        <v>1</v>
-      </c>
-      <c r="Y61">
+      <c r="W62">
+        <v>1</v>
+      </c>
+      <c r="X62" t="str">
+        <v/>
+      </c>
+      <c r="Y62">
         <v>650</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Y61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y62"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>